<commit_message>
feat: Add TGT Fulfillment Requests Line Item report and related functionality
</commit_message>
<xml_diff>
--- a/reports/tgt_fulfillment_params_requests/templates/xlsx/template.xlsx
+++ b/reports/tgt_fulfillment_params_requests/templates/xlsx/template.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Data!$AK$1:$AS$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Data!$A$1:$AK$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">Request ID</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t xml:space="preserve">Asset External ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset_Status</t>
   </si>
   <si>
     <t xml:space="preserve">Access_type</t>
@@ -239,12 +242,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -522,176 +529,179 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AS1"/>
+  <dimension ref="A1:AT1"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="3" min="3" style="0" width="19.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="4" min="4" style="0" width="14.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="6" min="5" style="0" width="17.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="8" min="8" style="0" width="10.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="9" style="0" width="18.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="22.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="23.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="26.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="18" style="0" width="18.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="26.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="26" style="0" width="18.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="0" width="18.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="15.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="20.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="15.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="13.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="14.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="24.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="22.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="0" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="0" width="19.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="0" width="17.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="3" min="3" style="1" width="19.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="4" min="4" style="1" width="14.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="6" min="5" style="1" width="17.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="8" min="8" style="1" width="10.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="9" style="1" width="18.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="22.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="23.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="26.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="19" style="1" width="18.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="26.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="27" style="1" width="18.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="34" style="1" width="18.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="15.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="20.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="15.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="13.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="14.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="24.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="22.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="19.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="17.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AG1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AH1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AI1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AK1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AL1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AM1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AN1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AO1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AP1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AR1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AS1" s="2" t="s">
         <v>44</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="AK1:AS1"/>
+  <autoFilter ref="A1:AK1"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
feat: Add TGT Fulfillment Requests Line Item report and related functionality (#51)
</commit_message>
<xml_diff>
--- a/reports/tgt_fulfillment_params_requests/templates/xlsx/template.xlsx
+++ b/reports/tgt_fulfillment_params_requests/templates/xlsx/template.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Data" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Data!$AK$1:$AS$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Data!$A$1:$AK$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">Request ID</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t xml:space="preserve">Asset External ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset_Status</t>
   </si>
   <si>
     <t xml:space="preserve">Access_type</t>
@@ -239,12 +242,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -522,176 +529,179 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AS1"/>
+  <dimension ref="A1:AT1"/>
   <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="1"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="3" min="3" style="0" width="19.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="4" min="4" style="0" width="14.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="6" min="5" style="0" width="17.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="8" min="8" style="0" width="10.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="9" style="0" width="18.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="22.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="23.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="26.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="18" style="0" width="18.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="26.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="26" style="0" width="18.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="0" width="18.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="35" style="0" width="15.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="0" width="20.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="0" width="15.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="0" width="13.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="0" width="14.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="0" width="24.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="0" width="22.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="0" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="0" width="19.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="0" width="17.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="3" min="3" style="1" width="19.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="4" min="4" style="1" width="14.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="6" min="5" style="1" width="17.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="1" max="8" min="8" style="1" width="10.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="9" style="1" width="18.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="22.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="23.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="26.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="19" style="1" width="18.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="26.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="27" style="1" width="18.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="35" min="34" style="1" width="18.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="15.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="20.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="15.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="13.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="14.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="24.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="22.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="19.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="17.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AG1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AH1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AI1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AK1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AL1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AM1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AN1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AO1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AP1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AR1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AS1" s="2" t="s">
         <v>44</v>
+      </c>
+      <c r="AT1" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="AK1:AS1"/>
+  <autoFilter ref="A1:AK1"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>